<commit_message>
Final QA: exclude US homeopathic listings from injectable share, utility wording, evidence text cleanup
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0172aZyF91urYrmsEU7SxkRE
</commit_message>
<xml_diff>
--- a/research/API_Injectable_Share.xlsx
+++ b/research/API_Injectable_Share.xlsx
@@ -1654,14 +1654,14 @@
         <v>0.0740740740740741</v>
       </c>
       <c r="V7" s="8" t="n">
-        <v>114</v>
+        <v>86</v>
       </c>
       <c r="W7" s="8" t="n">
         <v>12</v>
       </c>
       <c r="X7" s="10" t="n">
         <f aca="false">IF(V7&gt;=$C$3,W7/V7,"")</f>
-        <v>0.105263157894737</v>
+        <v>0.13953488372093</v>
       </c>
       <c r="Y7" s="8" t="n">
         <f aca="false">COUNT(F7,I7,L7,O7,R7,U7,X7)</f>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="Z7" s="11" t="n">
         <f aca="false">IF(Y7=0,"n/a",AVERAGE(F7,I7,L7,O7,R7,U7,X7))</f>
-        <v>0.673942003609456</v>
+        <v>0.679653957913821</v>
       </c>
       <c r="AA7" s="12" t="n">
         <f aca="false">IF(Y7=0,"",MIN(F7,I7,L7,O7,R7,U7,X7))</f>
@@ -1685,7 +1685,7 @@
       </c>
       <c r="AD7" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z7),C7*Z7,"")</f>
-        <v>2850.55227440681</v>
+        <v>2874.71195616935</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2599,14 +2599,14 @@
         <v>0.866666666666667</v>
       </c>
       <c r="V16" s="8" t="n">
-        <v>135</v>
+        <v>88</v>
       </c>
       <c r="W16" s="8" t="n">
         <v>53</v>
       </c>
       <c r="X16" s="10" t="n">
         <f aca="false">IF(V16&gt;=$C$3,W16/V16,"")</f>
-        <v>0.392592592592593</v>
+        <v>0.602272727272727</v>
       </c>
       <c r="Y16" s="8" t="n">
         <f aca="false">COUNT(F16,I16,L16,O16,R16,U16,X16)</f>
@@ -2614,11 +2614,11 @@
       </c>
       <c r="Z16" s="11" t="n">
         <f aca="false">IF(Y16=0,"n/a",AVERAGE(F16,I16,L16,O16,R16,U16,X16))</f>
-        <v>0.702152361952863</v>
+        <v>0.732106666907168</v>
       </c>
       <c r="AA16" s="12" t="n">
         <f aca="false">IF(Y16=0,"",MIN(F16,I16,L16,O16,R16,U16,X16))</f>
-        <v>0.392592592592593</v>
+        <v>0.541666666666667</v>
       </c>
       <c r="AB16" s="11" t="n">
         <f aca="false">IF(Y16=0,"",MAX(F16,I16,L16,O16,R16,U16,X16))</f>
@@ -2630,7 +2630,7 @@
       </c>
       <c r="AD16" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z16),C16*Z16,"")</f>
-        <v>6526.60450568253</v>
+        <v>6805.03396383549</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3439,14 +3439,14 @@
         <v>0.128205128205128</v>
       </c>
       <c r="V24" s="8" t="n">
-        <v>162</v>
+        <v>139</v>
       </c>
       <c r="W24" s="8" t="n">
         <v>9</v>
       </c>
       <c r="X24" s="10" t="n">
         <f aca="false">IF(V24&gt;=$C$3,W24/V24,"")</f>
-        <v>0.0555555555555556</v>
+        <v>0.0647482014388489</v>
       </c>
       <c r="Y24" s="8" t="n">
         <f aca="false">COUNT(F24,I24,L24,O24,R24,U24,X24)</f>
@@ -3454,7 +3454,7 @@
       </c>
       <c r="Z24" s="11" t="n">
         <f aca="false">IF(Y24=0,"n/a",AVERAGE(F24,I24,L24,O24,R24,U24,X24))</f>
-        <v>0.0511527360425806</v>
+        <v>0.0524659711687654</v>
       </c>
       <c r="AA24" s="12" t="n">
         <f aca="false">IF(Y24=0,"",MIN(F24,I24,L24,O24,R24,U24,X24))</f>
@@ -3470,7 +3470,7 @@
       </c>
       <c r="AD24" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z24),C24*Z24,"")</f>
-        <v>2557.09100243546</v>
+        <v>2622.7387465259</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4279,14 +4279,14 @@
         <v/>
       </c>
       <c r="V32" s="8" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="W32" s="8" t="n">
         <v>9</v>
       </c>
       <c r="X32" s="10" t="n">
         <f aca="false">IF(V32&gt;=$C$3,W32/V32,"")</f>
-        <v>0.136363636363636</v>
+        <v>0.140625</v>
       </c>
       <c r="Y32" s="8" t="n">
         <f aca="false">COUNT(F32,I32,L32,O32,R32,U32,X32)</f>
@@ -4294,7 +4294,7 @@
       </c>
       <c r="Z32" s="11" t="n">
         <f aca="false">IF(Y32=0,"n/a",AVERAGE(F32,I32,L32,O32,R32,U32,X32))</f>
-        <v>0.172727272727273</v>
+        <v>0.1734375</v>
       </c>
       <c r="AA32" s="12" t="n">
         <f aca="false">IF(Y32=0,"",MIN(F32,I32,L32,O32,R32,U32,X32))</f>
@@ -4310,7 +4310,7 @@
       </c>
       <c r="AD32" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z32),C32*Z32,"")</f>
-        <v>1352.64109090909</v>
+        <v>1358.2029375</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4594,14 +4594,14 @@
         <v>0.0434782608695652</v>
       </c>
       <c r="V35" s="8" t="n">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="W35" s="8" t="n">
         <v>17</v>
       </c>
       <c r="X35" s="10" t="n">
         <f aca="false">IF(V35&gt;=$C$3,W35/V35,"")</f>
-        <v>0.140495867768595</v>
+        <v>0.146551724137931</v>
       </c>
       <c r="Y35" s="8" t="n">
         <f aca="false">COUNT(F35,I35,L35,O35,R35,U35,X35)</f>
@@ -4609,7 +4609,7 @@
       </c>
       <c r="Z35" s="11" t="n">
         <f aca="false">IF(Y35=0,"n/a",AVERAGE(F35,I35,L35,O35,R35,U35,X35))</f>
-        <v>0.273441592608893</v>
+        <v>0.274306714947369</v>
       </c>
       <c r="AA35" s="12" t="n">
         <f aca="false">IF(Y35=0,"",MIN(F35,I35,L35,O35,R35,U35,X35))</f>
@@ -4625,7 +4625,7 @@
       </c>
       <c r="AD35" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z35),C35*Z35,"")</f>
-        <v>2405.42467394154</v>
+        <v>2413.03502538476</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6169,14 +6169,14 @@
         <v>0.909090909090909</v>
       </c>
       <c r="V50" s="8" t="n">
-        <v>218</v>
+        <v>90</v>
       </c>
       <c r="W50" s="8" t="n">
         <v>76</v>
       </c>
       <c r="X50" s="10" t="n">
         <f aca="false">IF(V50&gt;=$C$3,W50/V50,"")</f>
-        <v>0.348623853211009</v>
+        <v>0.844444444444444</v>
       </c>
       <c r="Y50" s="8" t="n">
         <f aca="false">COUNT(F50,I50,L50,O50,R50,U50,X50)</f>
@@ -6184,11 +6184,11 @@
       </c>
       <c r="Z50" s="11" t="n">
         <f aca="false">IF(Y50=0,"n/a",AVERAGE(F50,I50,L50,O50,R50,U50,X50))</f>
-        <v>0.805616176558289</v>
+        <v>0.876447689591637</v>
       </c>
       <c r="AA50" s="12" t="n">
         <f aca="false">IF(Y50=0,"",MIN(F50,I50,L50,O50,R50,U50,X50))</f>
-        <v>0.348623853211009</v>
+        <v>0.568181818181818</v>
       </c>
       <c r="AB50" s="11" t="n">
         <f aca="false">IF(Y50=0,"",MAX(F50,I50,L50,O50,R50,U50,X50))</f>
@@ -6196,11 +6196,11 @@
       </c>
       <c r="AC50" s="8" t="str">
         <f aca="false">IF(Y50&lt;2,"",IF(AB50-AA50&gt;$F$3,"Review",""))</f>
-        <v>Review</v>
+        <v/>
       </c>
       <c r="AD50" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z50),C50*Z50,"")</f>
-        <v>3722.26092600815</v>
+        <v>4049.5301405123</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8689,14 +8689,14 @@
         <v>1</v>
       </c>
       <c r="V74" s="8" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="W74" s="8" t="n">
         <v>17</v>
       </c>
       <c r="X74" s="10" t="n">
         <f aca="false">IF(V74&gt;=$C$3,W74/V74,"")</f>
-        <v>0.739130434782609</v>
+        <v>1</v>
       </c>
       <c r="Y74" s="8" t="n">
         <f aca="false">COUNT(F74,I74,L74,O74,R74,U74,X74)</f>
@@ -8704,11 +8704,11 @@
       </c>
       <c r="Z74" s="11" t="n">
         <f aca="false">IF(Y74=0,"n/a",AVERAGE(F74,I74,L74,O74,R74,U74,X74))</f>
-        <v>0.934782608695652</v>
+        <v>1</v>
       </c>
       <c r="AA74" s="12" t="n">
         <f aca="false">IF(Y74=0,"",MIN(F74,I74,L74,O74,R74,U74,X74))</f>
-        <v>0.739130434782609</v>
+        <v>1</v>
       </c>
       <c r="AB74" s="11" t="n">
         <f aca="false">IF(Y74=0,"",MAX(F74,I74,L74,O74,R74,U74,X74))</f>
@@ -8720,7 +8720,7 @@
       </c>
       <c r="AD74" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z74),C74*Z74,"")</f>
-        <v>163.643043478261</v>
+        <v>175.06</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8899,14 +8899,14 @@
         <v>0.173913043478261</v>
       </c>
       <c r="V76" s="8" t="n">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="W76" s="8" t="n">
         <v>7</v>
       </c>
       <c r="X76" s="10" t="n">
         <f aca="false">IF(V76&gt;=$C$3,W76/V76,"")</f>
-        <v>0.0330188679245283</v>
+        <v>0.0341463414634146</v>
       </c>
       <c r="Y76" s="8" t="n">
         <f aca="false">COUNT(F76,I76,L76,O76,R76,U76,X76)</f>
@@ -8914,11 +8914,11 @@
       </c>
       <c r="Z76" s="11" t="n">
         <f aca="false">IF(Y76=0,"n/a",AVERAGE(F76,I76,L76,O76,R76,U76,X76))</f>
-        <v>0.125714523309917</v>
+        <v>0.125875590958329</v>
       </c>
       <c r="AA76" s="12" t="n">
         <f aca="false">IF(Y76=0,"",MIN(F76,I76,L76,O76,R76,U76,X76))</f>
-        <v>0.0330188679245283</v>
+        <v>0.0341463414634146</v>
       </c>
       <c r="AB76" s="11" t="n">
         <f aca="false">IF(Y76=0,"",MAX(F76,I76,L76,O76,R76,U76,X76))</f>
@@ -8930,7 +8930,7 @@
       </c>
       <c r="AD76" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z76),C76*Z76,"")</f>
-        <v>4790.48642526433</v>
+        <v>4796.62408034947</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9109,7 +9109,7 @@
         <v/>
       </c>
       <c r="V78" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="W78" s="8" t="n">
         <v>0</v>
@@ -10054,14 +10054,14 @@
         <v>0.600917431192661</v>
       </c>
       <c r="V87" s="8" t="n">
-        <v>568</v>
+        <v>561</v>
       </c>
       <c r="W87" s="8" t="n">
         <v>105</v>
       </c>
       <c r="X87" s="10" t="n">
         <f aca="false">IF(V87&gt;=$C$3,W87/V87,"")</f>
-        <v>0.184859154929577</v>
+        <v>0.18716577540107</v>
       </c>
       <c r="Y87" s="8" t="n">
         <f aca="false">COUNT(F87,I87,L87,O87,R87,U87,X87)</f>
@@ -10069,11 +10069,11 @@
       </c>
       <c r="Z87" s="11" t="n">
         <f aca="false">IF(Y87=0,"n/a",AVERAGE(F87,I87,L87,O87,R87,U87,X87))</f>
-        <v>0.397871292803773</v>
+        <v>0.398200810013986</v>
       </c>
       <c r="AA87" s="12" t="n">
         <f aca="false">IF(Y87=0,"",MIN(F87,I87,L87,O87,R87,U87,X87))</f>
-        <v>0.184859154929577</v>
+        <v>0.18716577540107</v>
       </c>
       <c r="AB87" s="11" t="n">
         <f aca="false">IF(Y87=0,"",MAX(F87,I87,L87,O87,R87,U87,X87))</f>
@@ -10085,7 +10085,7 @@
       </c>
       <c r="AD87" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z87),C87*Z87,"")</f>
-        <v>18596.2137796046</v>
+        <v>18611.6151734624</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10264,14 +10264,14 @@
         <v>0.655172413793103</v>
       </c>
       <c r="V89" s="8" t="n">
-        <v>99</v>
+        <v>54</v>
       </c>
       <c r="W89" s="8" t="n">
         <v>33</v>
       </c>
       <c r="X89" s="10" t="n">
         <f aca="false">IF(V89&gt;=$C$3,W89/V89,"")</f>
-        <v>0.333333333333333</v>
+        <v>0.611111111111111</v>
       </c>
       <c r="Y89" s="8" t="n">
         <f aca="false">COUNT(F89,I89,L89,O89,R89,U89,X89)</f>
@@ -10279,11 +10279,11 @@
       </c>
       <c r="Z89" s="11" t="n">
         <f aca="false">IF(Y89=0,"n/a",AVERAGE(F89,I89,L89,O89,R89,U89,X89))</f>
-        <v>0.687931860654517</v>
+        <v>0.727614400337057</v>
       </c>
       <c r="AA89" s="12" t="n">
         <f aca="false">IF(Y89=0,"",MIN(F89,I89,L89,O89,R89,U89,X89))</f>
-        <v>0.333333333333333</v>
+        <v>0.383561643835616</v>
       </c>
       <c r="AB89" s="11" t="n">
         <f aca="false">IF(Y89=0,"",MAX(F89,I89,L89,O89,R89,U89,X89))</f>
@@ -10295,7 +10295,7 @@
       </c>
       <c r="AD89" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z89),C89*Z89,"")</f>
-        <v>11544.4253297947</v>
+        <v>12210.3519170963</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10369,26 +10369,26 @@
         <v>1</v>
       </c>
       <c r="V90" s="8" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="W90" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="X90" s="10" t="n">
+      <c r="X90" s="10" t="str">
         <f aca="false">IF(V90&gt;=$C$3,W90/V90,"")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Y90" s="8" t="n">
         <f aca="false">COUNT(F90,I90,L90,O90,R90,U90,X90)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Z90" s="11" t="n">
         <f aca="false">IF(Y90=0,"n/a",AVERAGE(F90,I90,L90,O90,R90,U90,X90))</f>
-        <v>0.857142857142857</v>
+        <v>1</v>
       </c>
       <c r="AA90" s="12" t="n">
         <f aca="false">IF(Y90=0,"",MIN(F90,I90,L90,O90,R90,U90,X90))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB90" s="11" t="n">
         <f aca="false">IF(Y90=0,"",MAX(F90,I90,L90,O90,R90,U90,X90))</f>
@@ -10396,11 +10396,11 @@
       </c>
       <c r="AC90" s="8" t="str">
         <f aca="false">IF(Y90&lt;2,"",IF(AB90-AA90&gt;$F$3,"Review",""))</f>
-        <v>Review</v>
+        <v/>
       </c>
       <c r="AD90" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z90),C90*Z90,"")</f>
-        <v>358084.465714286</v>
+        <v>417765.21</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11734,14 +11734,14 @@
         <v>0.857142857142857</v>
       </c>
       <c r="V103" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="W103" s="8" t="n">
         <v>27</v>
       </c>
       <c r="X103" s="10" t="n">
         <f aca="false">IF(V103&gt;=$C$3,W103/V103,"")</f>
-        <v>0.25</v>
+        <v>0.257142857142857</v>
       </c>
       <c r="Y103" s="8" t="n">
         <f aca="false">COUNT(F103,I103,L103,O103,R103,U103,X103)</f>
@@ -11749,11 +11749,11 @@
       </c>
       <c r="Z103" s="11" t="n">
         <f aca="false">IF(Y103=0,"n/a",AVERAGE(F103,I103,L103,O103,R103,U103,X103))</f>
-        <v>0.484908175406181</v>
+        <v>0.485928583569446</v>
       </c>
       <c r="AA103" s="12" t="n">
         <f aca="false">IF(Y103=0,"",MIN(F103,I103,L103,O103,R103,U103,X103))</f>
-        <v>0.25</v>
+        <v>0.257142857142857</v>
       </c>
       <c r="AB103" s="11" t="n">
         <f aca="false">IF(Y103=0,"",MAX(F103,I103,L103,O103,R103,U103,X103))</f>
@@ -11765,7 +11765,7 @@
       </c>
       <c r="AD103" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z103),C103*Z103,"")</f>
-        <v>1765.1287965413</v>
+        <v>1768.84321490865</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12574,14 +12574,14 @@
         <v>1</v>
       </c>
       <c r="V111" s="8" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="W111" s="8" t="n">
         <v>3</v>
       </c>
       <c r="X111" s="10" t="n">
         <f aca="false">IF(V111&gt;=$C$3,W111/V111,"")</f>
-        <v>0.157894736842105</v>
+        <v>1</v>
       </c>
       <c r="Y111" s="8" t="n">
         <f aca="false">COUNT(F111,I111,L111,O111,R111,U111,X111)</f>
@@ -12589,11 +12589,11 @@
       </c>
       <c r="Z111" s="11" t="n">
         <f aca="false">IF(Y111=0,"n/a",AVERAGE(F111,I111,L111,O111,R111,U111,X111))</f>
-        <v>0.863192645479244</v>
+        <v>0.983493397358944</v>
       </c>
       <c r="AA111" s="12" t="n">
         <f aca="false">IF(Y111=0,"",MIN(F111,I111,L111,O111,R111,U111,X111))</f>
-        <v>0.157894736842105</v>
+        <v>0.928571428571429</v>
       </c>
       <c r="AB111" s="11" t="n">
         <f aca="false">IF(Y111=0,"",MAX(F111,I111,L111,O111,R111,U111,X111))</f>
@@ -12601,11 +12601,11 @@
       </c>
       <c r="AC111" s="8" t="str">
         <f aca="false">IF(Y111&lt;2,"",IF(AB111-AA111&gt;$F$3,"Review",""))</f>
-        <v>Review</v>
+        <v/>
       </c>
       <c r="AD111" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z111),C111*Z111,"")</f>
-        <v>7218.2154358059</v>
+        <v>8224.19799219688</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13624,14 +13624,14 @@
         <v>0.0657894736842105</v>
       </c>
       <c r="V121" s="8" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="W121" s="8" t="n">
         <v>18</v>
       </c>
       <c r="X121" s="10" t="n">
         <f aca="false">IF(V121&gt;=$C$3,W121/V121,"")</f>
-        <v>0.72</v>
+        <v>0.782608695652174</v>
       </c>
       <c r="Y121" s="8" t="n">
         <f aca="false">COUNT(F121,I121,L121,O121,R121,U121,X121)</f>
@@ -13639,7 +13639,7 @@
       </c>
       <c r="Z121" s="11" t="n">
         <f aca="false">IF(Y121=0,"n/a",AVERAGE(F121,I121,L121,O121,R121,U121,X121))</f>
-        <v>0.455812270878129</v>
+        <v>0.468334010008564</v>
       </c>
       <c r="AA121" s="12" t="n">
         <f aca="false">IF(Y121=0,"",MIN(F121,I121,L121,O121,R121,U121,X121))</f>
@@ -13655,7 +13655,7 @@
       </c>
       <c r="AD121" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z121),C121*Z121,"")</f>
-        <v>2630.04591921222</v>
+        <v>2702.29660442962</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13939,14 +13939,14 @@
         <v>0.2</v>
       </c>
       <c r="V124" s="8" t="n">
-        <v>67</v>
+        <v>32</v>
       </c>
       <c r="W124" s="8" t="n">
         <v>4</v>
       </c>
       <c r="X124" s="10" t="n">
         <f aca="false">IF(V124&gt;=$C$3,W124/V124,"")</f>
-        <v>0.0597014925373134</v>
+        <v>0.125</v>
       </c>
       <c r="Y124" s="8" t="n">
         <f aca="false">COUNT(F124,I124,L124,O124,R124,U124,X124)</f>
@@ -13954,7 +13954,7 @@
       </c>
       <c r="Z124" s="11" t="n">
         <f aca="false">IF(Y124=0,"n/a",AVERAGE(F124,I124,L124,O124,R124,U124,X124))</f>
-        <v>0.110870072040337</v>
+        <v>0.120198430249293</v>
       </c>
       <c r="AA124" s="12" t="n">
         <f aca="false">IF(Y124=0,"",MIN(F124,I124,L124,O124,R124,U124,X124))</f>
@@ -13970,7 +13970,7 @@
       </c>
       <c r="AD124" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z124),C124*Z124,"")</f>
-        <v>2441.2270509425</v>
+        <v>2646.62639795743</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14884,14 +14884,14 @@
         <v>0.0416666666666667</v>
       </c>
       <c r="V133" s="8" t="n">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="W133" s="8" t="n">
         <v>34</v>
       </c>
       <c r="X133" s="10" t="n">
         <f aca="false">IF(V133&gt;=$C$3,W133/V133,"")</f>
-        <v>0.226666666666667</v>
+        <v>0.232876712328767</v>
       </c>
       <c r="Y133" s="8" t="n">
         <f aca="false">COUNT(F133,I133,L133,O133,R133,U133,X133)</f>
@@ -14899,7 +14899,7 @@
       </c>
       <c r="Z133" s="11" t="n">
         <f aca="false">IF(Y133=0,"n/a",AVERAGE(F133,I133,L133,O133,R133,U133,X133))</f>
-        <v>0.184745819777854</v>
+        <v>0.185632969158154</v>
       </c>
       <c r="AA133" s="12" t="n">
         <f aca="false">IF(Y133=0,"",MIN(F133,I133,L133,O133,R133,U133,X133))</f>
@@ -14915,7 +14915,7 @@
       </c>
       <c r="AD133" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z133),C133*Z133,"")</f>
-        <v>3633.2814951628</v>
+        <v>3650.72851199254</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14989,14 +14989,14 @@
         <v>0.285714285714286</v>
       </c>
       <c r="V134" s="8" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="W134" s="8" t="n">
         <v>4</v>
       </c>
       <c r="X134" s="10" t="n">
         <f aca="false">IF(V134&gt;=$C$3,W134/V134,"")</f>
-        <v>0.0547945205479452</v>
+        <v>0.0615384615384615</v>
       </c>
       <c r="Y134" s="8" t="n">
         <f aca="false">COUNT(F134,I134,L134,O134,R134,U134,X134)</f>
@@ -15004,7 +15004,7 @@
       </c>
       <c r="Z134" s="11" t="n">
         <f aca="false">IF(Y134=0,"n/a",AVERAGE(F134,I134,L134,O134,R134,U134,X134))</f>
-        <v>0.193196635159931</v>
+        <v>0.194160055301433</v>
       </c>
       <c r="AA134" s="12" t="n">
         <f aca="false">IF(Y134=0,"",MIN(F134,I134,L134,O134,R134,U134,X134))</f>
@@ -15020,7 +15020,7 @@
       </c>
       <c r="AD134" s="9" t="n">
         <f aca="false">IF(ISNUMBER(Z134),C134*Z134,"")</f>
-        <v>3562.44935403155</v>
+        <v>3580.21433973078</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17509,7 +17509,7 @@
         <v>242</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>48355</v>
+        <v>35740</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>